<commit_message>
Fig.6/Fig.7 (10 h) redrawn with CAT-50 robust (WAF=1.930782)
</commit_message>
<xml_diff>
--- a/figs/data/fig6_10h.xlsx
+++ b/figs/data/fig6_10h.xlsx
@@ -204,6 +204,49 @@
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22860">
               <a:solidFill>
+                <a:srgbClr val="8E8E93"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="4"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="8E8E93"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="8E8E93"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림6 10시간 (10분 단위)'!$C$2:$C$61</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림6 10시간 (10분 단위)'!$D$2:$D$61</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'그림6 10시간 (10분 단위)'!F1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22860">
+              <a:solidFill>
                 <a:srgbClr val="E3A33B"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
@@ -226,22 +269,22 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'그림6 10시간 (10분 단위)'!$C$2:$C$61</f>
+              <f>'그림6 10시간 (10분 단위)'!$E$2:$E$61</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'그림6 10시간 (10분 단위)'!$D$2:$D$61</f>
+              <f>'그림6 10시간 (10분 단위)'!$F$2:$F$61</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
-              <f>'그림6 10시간 (10분 단위)'!G1</f>
+              <f>'그림6 10시간 (10분 단위)'!I1</f>
             </strRef>
           </tx>
           <spPr>
@@ -262,12 +305,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'그림6 10시간 (10분 단위)'!$F$2:$F$3</f>
+              <f>'그림6 10시간 (10분 단위)'!$H$2:$H$3</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'그림6 10시간 (10분 단위)'!$G$2:$G$3</f>
+              <f>'그림6 10시간 (10분 단위)'!$I$2:$I$3</f>
             </numRef>
           </yVal>
         </ser>
@@ -348,7 +391,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>12</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -660,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -676,20 +719,30 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>CAT-50 (견고 설정) 시간(h)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-50 (견고 설정) 10분 구간 WAF</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>CAT-37 (기본값) 시간(h)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>CAT-37 (기본값) 10분 구간 WAF</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>전환 시간</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>워크로드 전환 (5.05시간)</t>
         </is>
@@ -706,12 +759,18 @@
         <v>0.0833</v>
       </c>
       <c r="D2" t="n">
+        <v>1.2694</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="F2" t="n">
         <v>1.4363</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>5.049</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -726,12 +785,18 @@
         <v>0.25</v>
       </c>
       <c r="D3" t="n">
+        <v>1.2454</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F3" t="n">
         <v>1.3533</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>5.049</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -746,6 +811,12 @@
         <v>0.4167</v>
       </c>
       <c r="D4" t="n">
+        <v>1.2425</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.4167</v>
+      </c>
+      <c r="F4" t="n">
         <v>1.3188</v>
       </c>
     </row>
@@ -760,24 +831,30 @@
         <v>0.5833</v>
       </c>
       <c r="D5" t="n">
+        <v>1.2404</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.5833</v>
+      </c>
+      <c r="F5" t="n">
         <v>1.3102</v>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="H5" s="1" t="inlineStr">
         <is>
           <t>정책</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>10시간 전체 WAF</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="J5" s="1" t="inlineStr">
         <is>
           <t>OLTP 구간</t>
         </is>
       </c>
-      <c r="I5" s="1" t="inlineStr">
+      <c r="K5" s="1" t="inlineStr">
         <is>
           <t>Varmail 구간</t>
         </is>
@@ -794,20 +871,26 @@
         <v>0.75</v>
       </c>
       <c r="D6" t="n">
+        <v>1.2387</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F6" t="n">
         <v>1.3056</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>iCAT-v4 (제안)</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>1.927</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
         <v>1.226</v>
       </c>
-      <c r="I6" t="n">
+      <c r="K6" t="n">
         <v>2.052</v>
       </c>
     </row>
@@ -822,35 +905,61 @@
         <v>0.9167</v>
       </c>
       <c r="D7" t="n">
+        <v>1.2374</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.9167</v>
+      </c>
+      <c r="F7" t="n">
         <v>1.3014</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>CAT-50 (견고 설정)</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>1.931</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.237</v>
+      </c>
+      <c r="K7" t="n">
+        <v>2.051</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1.0833</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1.216</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.0833</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.2373</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.0833</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.2916</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>CAT-37 (기본값)</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="I8" t="n">
         <v>2.122</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J8" t="n">
         <v>1.295</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K8" t="n">
         <v>2.336</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>1.0833</v>
-      </c>
-      <c r="B8" t="n">
-        <v>1.216</v>
-      </c>
-      <c r="C8" t="n">
-        <v>1.0833</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1.2916</v>
       </c>
     </row>
     <row r="9">
@@ -864,6 +973,12 @@
         <v>1.25</v>
       </c>
       <c r="D9" t="n">
+        <v>1.2387</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F9" t="n">
         <v>1.2902</v>
       </c>
     </row>
@@ -878,6 +993,12 @@
         <v>1.4167</v>
       </c>
       <c r="D10" t="n">
+        <v>1.2395</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.4167</v>
+      </c>
+      <c r="F10" t="n">
         <v>1.2908</v>
       </c>
     </row>
@@ -892,6 +1013,12 @@
         <v>1.5833</v>
       </c>
       <c r="D11" t="n">
+        <v>1.2339</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.5833</v>
+      </c>
+      <c r="F11" t="n">
         <v>1.285</v>
       </c>
     </row>
@@ -906,6 +1033,12 @@
         <v>1.75</v>
       </c>
       <c r="D12" t="n">
+        <v>1.2301</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F12" t="n">
         <v>1.2849</v>
       </c>
     </row>
@@ -920,6 +1053,12 @@
         <v>1.9167</v>
       </c>
       <c r="D13" t="n">
+        <v>1.2253</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.9167</v>
+      </c>
+      <c r="F13" t="n">
         <v>1.2872</v>
       </c>
     </row>
@@ -934,6 +1073,12 @@
         <v>2.0833</v>
       </c>
       <c r="D14" t="n">
+        <v>1.2345</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.0833</v>
+      </c>
+      <c r="F14" t="n">
         <v>1.2868</v>
       </c>
     </row>
@@ -948,6 +1093,12 @@
         <v>2.25</v>
       </c>
       <c r="D15" t="n">
+        <v>1.2359</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F15" t="n">
         <v>1.2864</v>
       </c>
     </row>
@@ -962,6 +1113,12 @@
         <v>2.4167</v>
       </c>
       <c r="D16" t="n">
+        <v>1.2369</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2.4167</v>
+      </c>
+      <c r="F16" t="n">
         <v>1.2858</v>
       </c>
     </row>
@@ -976,6 +1133,12 @@
         <v>2.5833</v>
       </c>
       <c r="D17" t="n">
+        <v>1.2354</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.5833</v>
+      </c>
+      <c r="F17" t="n">
         <v>1.2839</v>
       </c>
     </row>
@@ -990,6 +1153,12 @@
         <v>2.75</v>
       </c>
       <c r="D18" t="n">
+        <v>1.2353</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F18" t="n">
         <v>1.2841</v>
       </c>
     </row>
@@ -1004,6 +1173,12 @@
         <v>2.9167</v>
       </c>
       <c r="D19" t="n">
+        <v>1.2336</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.9167</v>
+      </c>
+      <c r="F19" t="n">
         <v>1.2833</v>
       </c>
     </row>
@@ -1018,6 +1193,12 @@
         <v>3.0833</v>
       </c>
       <c r="D20" t="n">
+        <v>1.2334</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.0833</v>
+      </c>
+      <c r="F20" t="n">
         <v>1.2821</v>
       </c>
     </row>
@@ -1032,6 +1213,12 @@
         <v>3.25</v>
       </c>
       <c r="D21" t="n">
+        <v>1.2345</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F21" t="n">
         <v>1.2814</v>
       </c>
     </row>
@@ -1046,6 +1233,12 @@
         <v>3.4167</v>
       </c>
       <c r="D22" t="n">
+        <v>1.2358</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.4167</v>
+      </c>
+      <c r="F22" t="n">
         <v>1.2817</v>
       </c>
     </row>
@@ -1060,6 +1253,12 @@
         <v>3.5833</v>
       </c>
       <c r="D23" t="n">
+        <v>1.2376</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3.5833</v>
+      </c>
+      <c r="F23" t="n">
         <v>1.281</v>
       </c>
     </row>
@@ -1074,6 +1273,12 @@
         <v>3.75</v>
       </c>
       <c r="D24" t="n">
+        <v>1.2341</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F24" t="n">
         <v>1.2795</v>
       </c>
     </row>
@@ -1088,6 +1293,12 @@
         <v>3.9167</v>
       </c>
       <c r="D25" t="n">
+        <v>1.2358</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3.9167</v>
+      </c>
+      <c r="F25" t="n">
         <v>1.2785</v>
       </c>
     </row>
@@ -1102,6 +1313,12 @@
         <v>4.0833</v>
       </c>
       <c r="D26" t="n">
+        <v>1.2394</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4.0833</v>
+      </c>
+      <c r="F26" t="n">
         <v>1.2795</v>
       </c>
     </row>
@@ -1116,6 +1333,12 @@
         <v>4.25</v>
       </c>
       <c r="D27" t="n">
+        <v>1.239</v>
+      </c>
+      <c r="E27" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F27" t="n">
         <v>1.2814</v>
       </c>
     </row>
@@ -1130,6 +1353,12 @@
         <v>4.4167</v>
       </c>
       <c r="D28" t="n">
+        <v>1.2377</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4.4167</v>
+      </c>
+      <c r="F28" t="n">
         <v>1.2822</v>
       </c>
     </row>
@@ -1144,6 +1373,12 @@
         <v>4.5833</v>
       </c>
       <c r="D29" t="n">
+        <v>1.2365</v>
+      </c>
+      <c r="E29" t="n">
+        <v>4.5833</v>
+      </c>
+      <c r="F29" t="n">
         <v>1.282</v>
       </c>
     </row>
@@ -1158,6 +1393,12 @@
         <v>4.75</v>
       </c>
       <c r="D30" t="n">
+        <v>1.2353</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="F30" t="n">
         <v>1.2822</v>
       </c>
     </row>
@@ -1172,6 +1413,12 @@
         <v>4.9167</v>
       </c>
       <c r="D31" t="n">
+        <v>1.2248</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4.9167</v>
+      </c>
+      <c r="F31" t="n">
         <v>1.2823</v>
       </c>
     </row>
@@ -1186,6 +1433,12 @@
         <v>5.0833</v>
       </c>
       <c r="D32" t="n">
+        <v>1.9548</v>
+      </c>
+      <c r="E32" t="n">
+        <v>5.0833</v>
+      </c>
+      <c r="F32" t="n">
         <v>2.3562</v>
       </c>
     </row>
@@ -1200,6 +1453,12 @@
         <v>5.25</v>
       </c>
       <c r="D33" t="n">
+        <v>2.051</v>
+      </c>
+      <c r="E33" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="F33" t="n">
         <v>2.4242</v>
       </c>
     </row>
@@ -1214,6 +1473,12 @@
         <v>5.4167</v>
       </c>
       <c r="D34" t="n">
+        <v>2.0518</v>
+      </c>
+      <c r="E34" t="n">
+        <v>5.4167</v>
+      </c>
+      <c r="F34" t="n">
         <v>2.4119</v>
       </c>
     </row>
@@ -1228,6 +1493,12 @@
         <v>5.5833</v>
       </c>
       <c r="D35" t="n">
+        <v>2.0512</v>
+      </c>
+      <c r="E35" t="n">
+        <v>5.5833</v>
+      </c>
+      <c r="F35" t="n">
         <v>2.404</v>
       </c>
     </row>
@@ -1242,6 +1513,12 @@
         <v>5.75</v>
       </c>
       <c r="D36" t="n">
+        <v>2.0513</v>
+      </c>
+      <c r="E36" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="F36" t="n">
         <v>2.3924</v>
       </c>
     </row>
@@ -1256,6 +1533,12 @@
         <v>5.9167</v>
       </c>
       <c r="D37" t="n">
+        <v>2.052</v>
+      </c>
+      <c r="E37" t="n">
+        <v>5.9167</v>
+      </c>
+      <c r="F37" t="n">
         <v>2.3846</v>
       </c>
     </row>
@@ -1270,6 +1553,12 @@
         <v>6.0833</v>
       </c>
       <c r="D38" t="n">
+        <v>2.0511</v>
+      </c>
+      <c r="E38" t="n">
+        <v>6.0833</v>
+      </c>
+      <c r="F38" t="n">
         <v>2.376</v>
       </c>
     </row>
@@ -1284,6 +1573,12 @@
         <v>6.25</v>
       </c>
       <c r="D39" t="n">
+        <v>2.0518</v>
+      </c>
+      <c r="E39" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F39" t="n">
         <v>2.3678</v>
       </c>
     </row>
@@ -1298,6 +1593,12 @@
         <v>6.4167</v>
       </c>
       <c r="D40" t="n">
+        <v>2.0514</v>
+      </c>
+      <c r="E40" t="n">
+        <v>6.4167</v>
+      </c>
+      <c r="F40" t="n">
         <v>2.3626</v>
       </c>
     </row>
@@ -1312,6 +1613,12 @@
         <v>6.5833</v>
       </c>
       <c r="D41" t="n">
+        <v>2.0514</v>
+      </c>
+      <c r="E41" t="n">
+        <v>6.5833</v>
+      </c>
+      <c r="F41" t="n">
         <v>2.3539</v>
       </c>
     </row>
@@ -1326,6 +1633,12 @@
         <v>6.75</v>
       </c>
       <c r="D42" t="n">
+        <v>2.0516</v>
+      </c>
+      <c r="E42" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="F42" t="n">
         <v>2.349</v>
       </c>
     </row>
@@ -1340,6 +1653,12 @@
         <v>6.9167</v>
       </c>
       <c r="D43" t="n">
+        <v>2.0509</v>
+      </c>
+      <c r="E43" t="n">
+        <v>6.9167</v>
+      </c>
+      <c r="F43" t="n">
         <v>2.342</v>
       </c>
     </row>
@@ -1354,6 +1673,12 @@
         <v>7.0833</v>
       </c>
       <c r="D44" t="n">
+        <v>2.0508</v>
+      </c>
+      <c r="E44" t="n">
+        <v>7.0833</v>
+      </c>
+      <c r="F44" t="n">
         <v>2.3377</v>
       </c>
     </row>
@@ -1368,6 +1693,12 @@
         <v>7.25</v>
       </c>
       <c r="D45" t="n">
+        <v>2.0511</v>
+      </c>
+      <c r="E45" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="F45" t="n">
         <v>2.3316</v>
       </c>
     </row>
@@ -1382,6 +1713,12 @@
         <v>7.4167</v>
       </c>
       <c r="D46" t="n">
+        <v>2.0511</v>
+      </c>
+      <c r="E46" t="n">
+        <v>7.4167</v>
+      </c>
+      <c r="F46" t="n">
         <v>2.3283</v>
       </c>
     </row>
@@ -1396,6 +1733,12 @@
         <v>7.5833</v>
       </c>
       <c r="D47" t="n">
+        <v>2.0511</v>
+      </c>
+      <c r="E47" t="n">
+        <v>7.5833</v>
+      </c>
+      <c r="F47" t="n">
         <v>2.324</v>
       </c>
     </row>
@@ -1410,6 +1753,12 @@
         <v>7.75</v>
       </c>
       <c r="D48" t="n">
+        <v>2.0517</v>
+      </c>
+      <c r="E48" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="F48" t="n">
         <v>2.318</v>
       </c>
     </row>
@@ -1424,6 +1773,12 @@
         <v>7.9167</v>
       </c>
       <c r="D49" t="n">
+        <v>2.0514</v>
+      </c>
+      <c r="E49" t="n">
+        <v>7.9167</v>
+      </c>
+      <c r="F49" t="n">
         <v>2.3153</v>
       </c>
     </row>
@@ -1438,6 +1793,12 @@
         <v>8.083299999999999</v>
       </c>
       <c r="D50" t="n">
+        <v>2.0503</v>
+      </c>
+      <c r="E50" t="n">
+        <v>8.083299999999999</v>
+      </c>
+      <c r="F50" t="n">
         <v>2.3127</v>
       </c>
     </row>
@@ -1452,6 +1813,12 @@
         <v>8.25</v>
       </c>
       <c r="D51" t="n">
+        <v>2.0511</v>
+      </c>
+      <c r="E51" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="F51" t="n">
         <v>2.3092</v>
       </c>
     </row>
@@ -1466,6 +1833,12 @@
         <v>8.416700000000001</v>
       </c>
       <c r="D52" t="n">
+        <v>2.0504</v>
+      </c>
+      <c r="E52" t="n">
+        <v>8.416700000000001</v>
+      </c>
+      <c r="F52" t="n">
         <v>2.3065</v>
       </c>
     </row>
@@ -1480,6 +1853,12 @@
         <v>8.583299999999999</v>
       </c>
       <c r="D53" t="n">
+        <v>2.0507</v>
+      </c>
+      <c r="E53" t="n">
+        <v>8.583299999999999</v>
+      </c>
+      <c r="F53" t="n">
         <v>2.3033</v>
       </c>
     </row>
@@ -1494,6 +1873,12 @@
         <v>8.75</v>
       </c>
       <c r="D54" t="n">
+        <v>2.0504</v>
+      </c>
+      <c r="E54" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="F54" t="n">
         <v>2.3012</v>
       </c>
     </row>
@@ -1508,6 +1893,12 @@
         <v>8.916700000000001</v>
       </c>
       <c r="D55" t="n">
+        <v>2.0505</v>
+      </c>
+      <c r="E55" t="n">
+        <v>8.916700000000001</v>
+      </c>
+      <c r="F55" t="n">
         <v>2.2972</v>
       </c>
     </row>
@@ -1522,6 +1913,12 @@
         <v>9.083299999999999</v>
       </c>
       <c r="D56" t="n">
+        <v>2.0507</v>
+      </c>
+      <c r="E56" t="n">
+        <v>9.083299999999999</v>
+      </c>
+      <c r="F56" t="n">
         <v>2.2966</v>
       </c>
     </row>
@@ -1536,6 +1933,12 @@
         <v>9.25</v>
       </c>
       <c r="D57" t="n">
+        <v>2.0503</v>
+      </c>
+      <c r="E57" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="F57" t="n">
         <v>2.2946</v>
       </c>
     </row>
@@ -1550,6 +1953,12 @@
         <v>9.416700000000001</v>
       </c>
       <c r="D58" t="n">
+        <v>2.0503</v>
+      </c>
+      <c r="E58" t="n">
+        <v>9.416700000000001</v>
+      </c>
+      <c r="F58" t="n">
         <v>2.293</v>
       </c>
     </row>
@@ -1564,6 +1973,12 @@
         <v>9.583299999999999</v>
       </c>
       <c r="D59" t="n">
+        <v>2.0515</v>
+      </c>
+      <c r="E59" t="n">
+        <v>9.583299999999999</v>
+      </c>
+      <c r="F59" t="n">
         <v>2.291</v>
       </c>
     </row>
@@ -1578,6 +1993,12 @@
         <v>9.75</v>
       </c>
       <c r="D60" t="n">
+        <v>2.0502</v>
+      </c>
+      <c r="E60" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="F60" t="n">
         <v>2.288</v>
       </c>
     </row>
@@ -1592,6 +2013,12 @@
         <v>9.916700000000001</v>
       </c>
       <c r="D61" t="n">
+        <v>2.0502</v>
+      </c>
+      <c r="E61" t="n">
+        <v>9.916700000000001</v>
+      </c>
+      <c r="F61" t="n">
         <v>2.2868</v>
       </c>
     </row>

</xml_diff>